<commit_message>
Fix cross-sheet formula references and DIV/0 error in FM template
</commit_message>
<xml_diff>
--- a/VisionVirtue_FM_Template.xlsx
+++ b/VisionVirtue_FM_Template.xlsx
@@ -5,7 +5,7 @@
   <sheets>
     <sheet name="Qualitative Assumptions" sheetId="1" r:id="rId1"/>
     <sheet name="Company Name P&amp;L" sheetId="2" r:id="rId2"/>
-    <sheet name="Company Name_Rev Build" sheetId="3" r:id="rId3"/>
+    <sheet name="Company Name Rev Build" sheetId="3" r:id="rId3"/>
     <sheet name="Company Name COGS+OPEX Build" sheetId="4" r:id="rId4"/>
     <sheet name="Capex Price Weighted AVG." sheetId="5" r:id="rId5"/>
   </sheets>
@@ -1275,27 +1275,27 @@
         <v>0.49130399999999996</v>
       </c>
       <c r="E3">
-        <f>'Neptune_Rev Build'!K36/1000</f>
+        <f>'Company Name Rev Build'!K36/1000</f>
         <v>0.4969159999999999</v>
       </c>
       <c r="F3">
-        <f>'Neptune_Rev Build'!O36/1000</f>
+        <f>'Company Name Rev Build'!O36/1000</f>
         <v>37.61136079999999</v>
       </c>
       <c r="G3">
-        <f>'Neptune_Rev Build'!S36/1000</f>
+        <f>'Company Name Rev Build'!S36/1000</f>
         <v>73.09314080000001</v>
       </c>
       <c r="H3">
-        <f>'Neptune_Rev Build'!W36/1000</f>
+        <f>'Company Name Rev Build'!W36/1000</f>
         <v>108.34965280000002</v>
       </c>
       <c r="I3">
-        <f>'Neptune_Rev Build'!AA36/1000</f>
+        <f>'Company Name Rev Build'!AA36/1000</f>
         <v>145.9632048</v>
       </c>
       <c r="J3">
-        <f>'Neptune_Rev Build'!AE36/1000</f>
+        <f>'Company Name Rev Build'!AE36/1000</f>
         <v>185.9337968</v>
       </c>
     </row>
@@ -1310,27 +1310,27 @@
         <v>0</v>
       </c>
       <c r="E4">
-        <f>'Neptune_Rev Build'!K39/1000</f>
+        <f>'Company Name Rev Build'!K39/1000</f>
         <v>0</v>
       </c>
       <c r="F4">
-        <f>'Neptune_Rev Build'!O39/1000</f>
+        <f>'Company Name Rev Build'!O39/1000</f>
         <v>0.258</v>
       </c>
       <c r="G4">
-        <f>'Neptune_Rev Build'!S39/1000</f>
+        <f>'Company Name Rev Build'!S39/1000</f>
         <v>1.95</v>
       </c>
       <c r="H4">
-        <f>'Neptune_Rev Build'!W39/1000</f>
+        <f>'Company Name Rev Build'!W39/1000</f>
         <v>4.422</v>
       </c>
       <c r="I4">
-        <f>'Neptune_Rev Build'!AA39/1000</f>
+        <f>'Company Name Rev Build'!AA39/1000</f>
         <v>7.674</v>
       </c>
       <c r="J4">
-        <f>'Neptune_Rev Build'!AE39/1000</f>
+        <f>'Company Name Rev Build'!AE39/1000</f>
         <v>11.706</v>
       </c>
     </row>
@@ -1345,27 +1345,27 @@
         <v>1.25</v>
       </c>
       <c r="E5">
-        <f>SUM('Neptune_Rev Build'!K51:K53)/1000</f>
+        <f>SUM('Company Name Rev Build'!K51:K53)/1000</f>
         <v>0.798</v>
       </c>
       <c r="F5">
-        <f>SUM('Neptune_Rev Build'!O51:O53)/1000</f>
+        <f>SUM('Company Name Rev Build'!O51:O53)/1000</f>
         <v>7.816</v>
       </c>
       <c r="G5">
-        <f>SUM('Neptune_Rev Build'!S51:S53)/1000</f>
+        <f>SUM('Company Name Rev Build'!S51:S53)/1000</f>
         <v>11.316</v>
       </c>
       <c r="H5">
-        <f>SUM('Neptune_Rev Build'!W51:W53)/1000</f>
+        <f>SUM('Company Name Rev Build'!W51:W53)/1000</f>
         <v>14.816</v>
       </c>
       <c r="I5">
-        <f>SUM('Neptune_Rev Build'!AA51:AA53)/1000</f>
+        <f>SUM('Company Name Rev Build'!AA51:AA53)/1000</f>
         <v>18.316</v>
       </c>
       <c r="J5">
-        <f>SUM('Neptune_Rev Build'!AE51:AE53)/1000</f>
+        <f>SUM('Company Name Rev Build'!AE51:AE53)/1000</f>
         <v>21.816</v>
       </c>
     </row>
@@ -1380,27 +1380,27 @@
         <v>10.5</v>
       </c>
       <c r="E6">
-        <f>('Neptune_Rev Build'!K55)/1000</f>
+        <f>('Company Name Rev Build'!K55)/1000</f>
         <v>10.432</v>
       </c>
       <c r="F6">
-        <f>('Neptune_Rev Build'!O55)/1000</f>
+        <f>('Company Name Rev Build'!O55)/1000</f>
         <v>12.373</v>
       </c>
       <c r="G6">
-        <f>('Neptune_Rev Build'!S55)/1000</f>
+        <f>('Company Name Rev Build'!S55)/1000</f>
         <v>13.373</v>
       </c>
       <c r="H6">
-        <f>('Neptune_Rev Build'!W55)/1000</f>
+        <f>('Company Name Rev Build'!W55)/1000</f>
         <v>14.373</v>
       </c>
       <c r="I6">
-        <f>('Neptune_Rev Build'!AA55)/1000</f>
+        <f>('Company Name Rev Build'!AA55)/1000</f>
         <v>15.373</v>
       </c>
       <c r="J6">
-        <f>('Neptune_Rev Build'!AE55)/1000</f>
+        <f>('Company Name Rev Build'!AE55)/1000</f>
         <v>16.373</v>
       </c>
     </row>
@@ -1415,27 +1415,27 @@
         <v>1.5</v>
       </c>
       <c r="E7">
-        <f>'Neptune_Rev Build'!K49/1000</f>
+        <f>'Company Name Rev Build'!K49/1000</f>
         <v>0.445</v>
       </c>
       <c r="F7">
-        <f>'Neptune_Rev Build'!O49/1000</f>
+        <f>'Company Name Rev Build'!O49/1000</f>
         <v>1.508</v>
       </c>
       <c r="G7">
-        <f>'Neptune_Rev Build'!S49/1000</f>
+        <f>'Company Name Rev Build'!S49/1000</f>
         <v>4.233</v>
       </c>
       <c r="H7">
-        <f>'Neptune_Rev Build'!W49/1000</f>
+        <f>'Company Name Rev Build'!W49/1000</f>
         <v>7.12675</v>
       </c>
       <c r="I7">
-        <f>'Neptune_Rev Build'!AA49/1000</f>
+        <f>'Company Name Rev Build'!AA49/1000</f>
         <v>10.3158125</v>
       </c>
       <c r="J7">
-        <f>'Neptune_Rev Build'!AE49/1000</f>
+        <f>'Company Name Rev Build'!AE49/1000</f>
         <v>14.021671875</v>
       </c>
     </row>
@@ -1525,27 +1525,27 @@
         <v>-8.746694377499999</v>
       </c>
       <c r="E11">
-        <f>-'Neptune COGS+OPEX Build'!M145</f>
+        <f>-'Company Name COGS+OPEX Build'!M145</f>
         <v>0</v>
       </c>
       <c r="F11">
-        <f>-'Neptune COGS+OPEX Build'!N145</f>
+        <f>-'Company Name COGS+OPEX Build'!N145</f>
         <v>-0.179</v>
       </c>
       <c r="G11">
-        <f>-'Neptune COGS+OPEX Build'!O145</f>
+        <f>-'Company Name COGS+OPEX Build'!O145</f>
         <v>-0.5982999999999998</v>
       </c>
       <c r="H11">
-        <f>-'Neptune COGS+OPEX Build'!P145</f>
+        <f>-'Company Name COGS+OPEX Build'!P145</f>
         <v>-0.8482999999999998</v>
       </c>
       <c r="I11">
-        <f>-'Neptune COGS+OPEX Build'!Q145</f>
+        <f>-'Company Name COGS+OPEX Build'!Q145</f>
         <v>-1.0982999999999998</v>
       </c>
       <c r="J11">
-        <f>-'Neptune COGS+OPEX Build'!R145</f>
+        <f>-'Company Name COGS+OPEX Build'!R145</f>
         <v>-1.3482999999999998</v>
       </c>
     </row>
@@ -1560,27 +1560,27 @@
         <v>-8.54</v>
       </c>
       <c r="E12">
-        <f>-'Neptune COGS+OPEX Build'!M191</f>
+        <f>-'Company Name COGS+OPEX Build'!M191</f>
         <v>-7.141</v>
       </c>
       <c r="F12">
-        <f>-'Neptune COGS+OPEX Build'!N191</f>
+        <f>-'Company Name COGS+OPEX Build'!N191</f>
         <v>-8.522</v>
       </c>
       <c r="G12">
-        <f>-'Neptune COGS+OPEX Build'!O191</f>
+        <f>-'Company Name COGS+OPEX Build'!O191</f>
         <v>-9.1181429890318</v>
       </c>
       <c r="H12">
-        <f>-'Neptune COGS+OPEX Build'!P191</f>
+        <f>-'Company Name COGS+OPEX Build'!P191</f>
         <v>-9.769588727166022</v>
       </c>
       <c r="I12">
-        <f>-'Neptune COGS+OPEX Build'!Q191</f>
+        <f>-'Company Name COGS+OPEX Build'!Q191</f>
         <v>-10.542090677632196</v>
       </c>
       <c r="J12">
-        <f>-'Neptune COGS+OPEX Build'!R191</f>
+        <f>-'Company Name COGS+OPEX Build'!R191</f>
         <v>-11.547783862710729</v>
       </c>
     </row>
@@ -1630,27 +1630,27 @@
         <v>-0.165</v>
       </c>
       <c r="E14">
-        <f>-'Neptune COGS+OPEX Build'!M175</f>
+        <f>-'Company Name COGS+OPEX Build'!M175</f>
         <v>-0.159</v>
       </c>
       <c r="F14">
-        <f>-'Neptune COGS+OPEX Build'!N175</f>
+        <f>-'Company Name COGS+OPEX Build'!N175</f>
         <v>-0.8440714285714286</v>
       </c>
       <c r="G14">
-        <f>-'Neptune COGS+OPEX Build'!O175</f>
+        <f>-'Company Name COGS+OPEX Build'!O175</f>
         <v>-1.6622142857142856</v>
       </c>
       <c r="H14">
-        <f>-'Neptune COGS+OPEX Build'!P175</f>
+        <f>-'Company Name COGS+OPEX Build'!P175</f>
         <v>-2.5542857142857147</v>
       </c>
       <c r="I14">
-        <f>-'Neptune COGS+OPEX Build'!Q175</f>
+        <f>-'Company Name COGS+OPEX Build'!Q175</f>
         <v>-3.8828571428571426</v>
       </c>
       <c r="J14">
-        <f>-'Neptune COGS+OPEX Build'!R175</f>
+        <f>-'Company Name COGS+OPEX Build'!R175</f>
         <v>-5.468571428571429</v>
       </c>
     </row>
@@ -1665,27 +1665,27 @@
         <v>-0.24</v>
       </c>
       <c r="E15">
-        <f>-'Neptune COGS+OPEX Build'!M176</f>
+        <f>-'Company Name COGS+OPEX Build'!M176</f>
         <v>-0.312</v>
       </c>
       <c r="F15">
-        <f>-'Neptune COGS+OPEX Build'!N176</f>
+        <f>-'Company Name COGS+OPEX Build'!N176</f>
         <v>-14.6265</v>
       </c>
       <c r="G15">
-        <f>-'Neptune COGS+OPEX Build'!O176</f>
+        <f>-'Company Name COGS+OPEX Build'!O176</f>
         <v>-14.94</v>
       </c>
       <c r="H15">
-        <f>-'Neptune COGS+OPEX Build'!P176</f>
+        <f>-'Company Name COGS+OPEX Build'!P176</f>
         <v>-17.94</v>
       </c>
       <c r="I15">
-        <f>-'Neptune COGS+OPEX Build'!Q176</f>
+        <f>-'Company Name COGS+OPEX Build'!Q176</f>
         <v>-20.94</v>
       </c>
       <c r="J15">
-        <f>-'Neptune COGS+OPEX Build'!R176</f>
+        <f>-'Company Name COGS+OPEX Build'!R176</f>
         <v>-23.94</v>
       </c>
     </row>
@@ -1700,27 +1700,27 @@
         <v>0</v>
       </c>
       <c r="E16">
-        <f>-'Neptune COGS+OPEX Build'!M177</f>
+        <f>-'Company Name COGS+OPEX Build'!M177</f>
         <v>-0.014907479999999997</v>
       </c>
       <c r="F16">
-        <f>-'Neptune COGS+OPEX Build'!N177</f>
+        <f>-'Company Name COGS+OPEX Build'!N177</f>
         <v>-1.1360808239999998</v>
       </c>
       <c r="G16">
-        <f>-'Neptune COGS+OPEX Build'!O177</f>
+        <f>-'Company Name COGS+OPEX Build'!O177</f>
         <v>-2.251294224</v>
       </c>
       <c r="H16">
-        <f>-'Neptune COGS+OPEX Build'!P177</f>
+        <f>-'Company Name COGS+OPEX Build'!P177</f>
         <v>-3.3831495840000003</v>
       </c>
       <c r="I16">
-        <f>-'Neptune COGS+OPEX Build'!Q177</f>
+        <f>-'Company Name COGS+OPEX Build'!Q177</f>
         <v>-4.609116144</v>
       </c>
       <c r="J16">
-        <f>-'Neptune COGS+OPEX Build'!R177</f>
+        <f>-'Company Name COGS+OPEX Build'!R177</f>
         <v>-5.929193904</v>
       </c>
     </row>
@@ -1770,27 +1770,27 @@
         <v>-18.43883723464285</v>
       </c>
       <c r="E18">
-        <f>-'Neptune COGS+OPEX Build'!M205</f>
+        <f>-'Company Name COGS+OPEX Build'!M205</f>
         <v>-11.502</v>
       </c>
       <c r="F18">
-        <f>-'Neptune COGS+OPEX Build'!N205</f>
+        <f>-'Company Name COGS+OPEX Build'!N205</f>
         <v>-38.129</v>
       </c>
       <c r="G18">
-        <f>-'Neptune COGS+OPEX Build'!O205</f>
+        <f>-'Company Name COGS+OPEX Build'!O205</f>
         <v>-46.95321236005971</v>
       </c>
       <c r="H18">
-        <f>-'Neptune COGS+OPEX Build'!P205</f>
+        <f>-'Company Name COGS+OPEX Build'!P205</f>
         <v>-58.41023752564013</v>
       </c>
       <c r="I18">
-        <f>-'Neptune COGS+OPEX Build'!Q205</f>
+        <f>-'Company Name COGS+OPEX Build'!Q205</f>
         <v>-70.53047744127186</v>
       </c>
       <c r="J18">
-        <f>-'Neptune COGS+OPEX Build'!R205</f>
+        <f>-'Company Name COGS+OPEX Build'!R205</f>
         <v>-83.23277104503809</v>
       </c>
     </row>
@@ -1875,27 +1875,27 @@
         <v>-4.3830056840000005</v>
       </c>
       <c r="E23">
-        <f>-'Neptune COGS+OPEX Build'!M40</f>
+        <f>-'Company Name COGS+OPEX Build'!M40</f>
         <v>-7.402660874666666</v>
       </c>
       <c r="F23">
-        <f>-'Neptune COGS+OPEX Build'!N40</f>
+        <f>-'Company Name COGS+OPEX Build'!N40</f>
         <v>-16.528202166186663</v>
       </c>
       <c r="G23">
-        <f>-'Neptune COGS+OPEX Build'!O40</f>
+        <f>-'Company Name COGS+OPEX Build'!O40</f>
         <v>-19.57862982104482</v>
       </c>
       <c r="H23">
-        <f>-'Neptune COGS+OPEX Build'!P40</f>
+        <f>-'Company Name COGS+OPEX Build'!P40</f>
         <v>-22.03347668350245</v>
       </c>
       <c r="I23">
-        <f>-'Neptune COGS+OPEX Build'!Q40</f>
+        <f>-'Company Name COGS+OPEX Build'!Q40</f>
         <v>-24.50141174885609</v>
       </c>
       <c r="J23">
-        <f>-'Neptune COGS+OPEX Build'!R40</f>
+        <f>-'Company Name COGS+OPEX Build'!R40</f>
         <v>-26.989853289392634</v>
       </c>
     </row>
@@ -1945,27 +1945,27 @@
         <v>-23.288410330625005</v>
       </c>
       <c r="E25">
-        <f>-'Neptune COGS+OPEX Build'!M129</f>
+        <f>-'Company Name COGS+OPEX Build'!M129</f>
         <v>-17.16984161066667</v>
       </c>
       <c r="F25">
-        <f>-'Neptune COGS+OPEX Build'!N129</f>
+        <f>-'Company Name COGS+OPEX Build'!N129</f>
         <v>-20.69119636288</v>
       </c>
       <c r="G25">
-        <f>-'Neptune COGS+OPEX Build'!O129</f>
+        <f>-'Company Name COGS+OPEX Build'!O129</f>
         <v>-21.61319059273211</v>
       </c>
       <c r="H25">
-        <f>-'Neptune COGS+OPEX Build'!P129</f>
+        <f>-'Company Name COGS+OPEX Build'!P129</f>
         <v>-22.57298832067987</v>
       </c>
       <c r="I25">
-        <f>-'Neptune COGS+OPEX Build'!Q129</f>
+        <f>-'Company Name COGS+OPEX Build'!Q129</f>
         <v>-23.470266597401515</v>
       </c>
       <c r="J25">
-        <f>-'Neptune COGS+OPEX Build'!R129</f>
+        <f>-'Company Name COGS+OPEX Build'!R129</f>
         <v>-24.61870989698702</v>
       </c>
     </row>
@@ -2015,27 +2015,27 @@
         <v>-20.930979095625</v>
       </c>
       <c r="E27">
-        <f>-'Neptune COGS+OPEX Build'!M74</f>
+        <f>-'Company Name COGS+OPEX Build'!M74</f>
         <v>-20.472702888</v>
       </c>
       <c r="F27">
-        <f>-'Neptune COGS+OPEX Build'!N74</f>
+        <f>-'Company Name COGS+OPEX Build'!N74</f>
         <v>-23.36587172896</v>
       </c>
       <c r="G27">
-        <f>-'Neptune COGS+OPEX Build'!O74</f>
+        <f>-'Company Name COGS+OPEX Build'!O74</f>
         <v>-24.975894779057278</v>
       </c>
       <c r="H27">
-        <f>-'Neptune COGS+OPEX Build'!P74</f>
+        <f>-'Company Name COGS+OPEX Build'!P74</f>
         <v>-25.21141622283114</v>
       </c>
       <c r="I27">
-        <f>-'Neptune COGS+OPEX Build'!Q74</f>
+        <f>-'Company Name COGS+OPEX Build'!Q74</f>
         <v>-25.618464089747683</v>
       </c>
       <c r="J27">
-        <f>-'Neptune COGS+OPEX Build'!R74</f>
+        <f>-'Company Name COGS+OPEX Build'!R74</f>
         <v>-26.332085368439188</v>
       </c>
     </row>
@@ -2192,27 +2192,27 @@
         <v>11.921</v>
       </c>
       <c r="E35">
-        <f>'Neptune COGS+OPEX Build'!M33+'Neptune COGS+OPEX Build'!M32+'Neptune COGS+OPEX Build'!M67+'Neptune COGS+OPEX Build'!M124</f>
+        <f>'Company Name COGS+OPEX Build'!M33+'Company Name COGS+OPEX Build'!M32+'Company Name COGS+OPEX Build'!M67+'Company Name COGS+OPEX Build'!M124</f>
         <v>1.49594228</v>
       </c>
       <c r="F35">
-        <f>'Neptune COGS+OPEX Build'!N33+'Neptune COGS+OPEX Build'!N32+'Neptune COGS+OPEX Build'!N67+'Neptune COGS+OPEX Build'!N124</f>
+        <f>'Company Name COGS+OPEX Build'!N33+'Company Name COGS+OPEX Build'!N32+'Company Name COGS+OPEX Build'!N67+'Company Name COGS+OPEX Build'!N124</f>
         <v>1.49594228</v>
       </c>
       <c r="G35">
-        <f>'Neptune COGS+OPEX Build'!O33+'Neptune COGS+OPEX Build'!O32+'Neptune COGS+OPEX Build'!O67+'Neptune COGS+OPEX Build'!O124</f>
+        <f>'Company Name COGS+OPEX Build'!O33+'Company Name COGS+OPEX Build'!O32+'Company Name COGS+OPEX Build'!O67+'Company Name COGS+OPEX Build'!O124</f>
         <v>1.49594228</v>
       </c>
       <c r="H35">
-        <f>'Neptune COGS+OPEX Build'!P33+'Neptune COGS+OPEX Build'!P32+'Neptune COGS+OPEX Build'!P67+'Neptune COGS+OPEX Build'!P124</f>
+        <f>'Company Name COGS+OPEX Build'!P33+'Company Name COGS+OPEX Build'!P32+'Company Name COGS+OPEX Build'!P67+'Company Name COGS+OPEX Build'!P124</f>
         <v>1.49594228</v>
       </c>
       <c r="I35">
-        <f>'Neptune COGS+OPEX Build'!Q33+'Neptune COGS+OPEX Build'!Q32+'Neptune COGS+OPEX Build'!Q67+'Neptune COGS+OPEX Build'!Q124</f>
+        <f>'Company Name COGS+OPEX Build'!Q33+'Company Name COGS+OPEX Build'!Q32+'Company Name COGS+OPEX Build'!Q67+'Company Name COGS+OPEX Build'!Q124</f>
         <v>1.49594228</v>
       </c>
       <c r="J35">
-        <f>'Neptune COGS+OPEX Build'!R33+'Neptune COGS+OPEX Build'!R32+'Neptune COGS+OPEX Build'!R67+'Neptune COGS+OPEX Build'!R124</f>
+        <f>'Company Name COGS+OPEX Build'!R33+'Company Name COGS+OPEX Build'!R32+'Company Name COGS+OPEX Build'!R67+'Company Name COGS+OPEX Build'!R124</f>
         <v>1.49594228</v>
       </c>
     </row>
@@ -2297,27 +2297,27 @@
         <v>5.9079999999999995</v>
       </c>
       <c r="E40">
-        <f>'Neptune COGS+OPEX Build'!M34++'Neptune COGS+OPEX Build'!M68+'Neptune COGS+OPEX Build'!M125+'Neptune COGS+OPEX Build'!M199</f>
+        <f>'Company Name COGS+OPEX Build'!M34++'Company Name COGS+OPEX Build'!M68+'Company Name COGS+OPEX Build'!M125+'Company Name COGS+OPEX Build'!M199</f>
         <v>6.6272666666666655</v>
       </c>
       <c r="F40">
-        <f>'Neptune COGS+OPEX Build'!N34++'Neptune COGS+OPEX Build'!N68+'Neptune COGS+OPEX Build'!N125+'Neptune COGS+OPEX Build'!N199</f>
+        <f>'Company Name COGS+OPEX Build'!N34++'Company Name COGS+OPEX Build'!N68+'Company Name COGS+OPEX Build'!N125+'Company Name COGS+OPEX Build'!N199</f>
         <v>9.450396666666665</v>
       </c>
       <c r="G40">
-        <f>'Neptune COGS+OPEX Build'!O34++'Neptune COGS+OPEX Build'!O68+'Neptune COGS+OPEX Build'!O125+'Neptune COGS+OPEX Build'!O199</f>
+        <f>'Company Name COGS+OPEX Build'!O34++'Company Name COGS+OPEX Build'!O68+'Company Name COGS+OPEX Build'!O125+'Company Name COGS+OPEX Build'!O199</f>
         <v>9.885749833333332</v>
       </c>
       <c r="H40">
-        <f>'Neptune COGS+OPEX Build'!P34++'Neptune COGS+OPEX Build'!P68+'Neptune COGS+OPEX Build'!P125+'Neptune COGS+OPEX Build'!P199</f>
+        <f>'Company Name COGS+OPEX Build'!P34++'Company Name COGS+OPEX Build'!P68+'Company Name COGS+OPEX Build'!P125+'Company Name COGS+OPEX Build'!P199</f>
         <v>10.241687324999997</v>
       </c>
       <c r="I40">
-        <f>'Neptune COGS+OPEX Build'!Q34++'Neptune COGS+OPEX Build'!Q68+'Neptune COGS+OPEX Build'!Q125+'Neptune COGS+OPEX Build'!Q199</f>
+        <f>'Company Name COGS+OPEX Build'!Q34++'Company Name COGS+OPEX Build'!Q68+'Company Name COGS+OPEX Build'!Q125+'Company Name COGS+OPEX Build'!Q199</f>
         <v>10.518238357916664</v>
       </c>
       <c r="J40">
-        <f>'Neptune COGS+OPEX Build'!R34++'Neptune COGS+OPEX Build'!R68+'Neptune COGS+OPEX Build'!R125+'Neptune COGS+OPEX Build'!R199</f>
+        <f>'Company Name COGS+OPEX Build'!R34++'Company Name COGS+OPEX Build'!R68+'Company Name COGS+OPEX Build'!R125+'Company Name COGS+OPEX Build'!R199</f>
         <v>10.715433609145832</v>
       </c>
     </row>
@@ -9830,27 +9830,27 @@
         <v>AI Rev.</v>
       </c>
       <c r="M147">
-        <f>'Neptune_Rev Build'!K51/1000</f>
+        <f>'Company Name Rev Build'!K51/1000</f>
         <v>0.798</v>
       </c>
       <c r="N147">
-        <f>'Neptune_Rev Build'!O51/1000</f>
+        <f>'Company Name Rev Build'!O51/1000</f>
         <v>3.483</v>
       </c>
       <c r="O147">
-        <f>'Neptune_Rev Build'!S51/1000</f>
+        <f>'Company Name Rev Build'!S51/1000</f>
         <v>5.983</v>
       </c>
       <c r="P147">
-        <f>'Neptune_Rev Build'!W51/1000</f>
+        <f>'Company Name Rev Build'!W51/1000</f>
         <v>8.483</v>
       </c>
       <c r="Q147">
-        <f>'Neptune_Rev Build'!AA51/1000</f>
+        <f>'Company Name Rev Build'!AA51/1000</f>
         <v>10.983</v>
       </c>
       <c r="R147">
-        <f>'Neptune_Rev Build'!AE51/1000</f>
+        <f>'Company Name Rev Build'!AE51/1000</f>
         <v>13.483</v>
       </c>
     </row>
@@ -10064,9 +10064,9 @@
       <c r="J156" t="str">
         <v>[Acquisition] GM.</v>
       </c>
-      <c r="M156" t="e">
-        <f>(M157-M155)/M157</f>
-        <v>#DIV/0!</v>
+      <c r="M156">
+        <f>IFERROR((M157-M155)/M157,0)</f>
+        <v>0</v>
       </c>
       <c r="N156">
         <f>(N157-N155)/N157</f>
@@ -10094,27 +10094,27 @@
         <v>[Acquisition] Rev.</v>
       </c>
       <c r="M157">
-        <f>'Neptune_Rev Build'!K53/1000</f>
+        <f>'Company Name Rev Build'!K53/1000</f>
         <v>0</v>
       </c>
       <c r="N157">
-        <f>'Neptune_Rev Build'!O53/1000</f>
+        <f>'Company Name Rev Build'!O53/1000</f>
         <v>4.333</v>
       </c>
       <c r="O157">
-        <f>'Neptune_Rev Build'!S53/1000</f>
+        <f>'Company Name Rev Build'!S53/1000</f>
         <v>5.333</v>
       </c>
       <c r="P157">
-        <f>'Neptune_Rev Build'!W53/1000</f>
+        <f>'Company Name Rev Build'!W53/1000</f>
         <v>6.333</v>
       </c>
       <c r="Q157">
-        <f>'Neptune_Rev Build'!AA53/1000</f>
+        <f>'Company Name Rev Build'!AA53/1000</f>
         <v>7.333</v>
       </c>
       <c r="R157">
-        <f>'Neptune_Rev Build'!AE53/1000</f>
+        <f>'Company Name Rev Build'!AE53/1000</f>
         <v>8.333</v>
       </c>
     </row>
@@ -10421,23 +10421,23 @@
         <v>0</v>
       </c>
       <c r="N171">
-        <f>(AVERAGE('Neptune_Rev Build'!M7,'Neptune_Rev Build'!I7)*('Neptune_Rev Build'!M18*'Neptune_Rev Build'!M19)*12*'Neptune COGS+OPEX Build'!$E$171)/1000000</f>
+        <f>(AVERAGE('Company Name Rev Build'!M7,'Company Name Rev Build'!I7)*('Company Name Rev Build'!M18*'Company Name Rev Build'!M19)*12*'Company Name COGS+OPEX Build'!$E$171)/1000000</f>
         <v>1.6200647999999995</v>
       </c>
       <c r="O171">
-        <f>(AVERAGE('Neptune_Rev Build'!M7,'Neptune_Rev Build'!Q7)*('Neptune_Rev Build'!Q18*'Neptune_Rev Build'!Q19)*12*'Neptune COGS+OPEX Build'!$E$171)/1000000</f>
+        <f>(AVERAGE('Company Name Rev Build'!M7,'Company Name Rev Build'!Q7)*('Company Name Rev Build'!Q18*'Company Name Rev Build'!Q19)*12*'Company Name COGS+OPEX Build'!$E$171)/1000000</f>
         <v>4.8600648</v>
       </c>
       <c r="P171">
-        <f>(AVERAGE('Neptune_Rev Build'!Q7,'Neptune_Rev Build'!U7)*('Neptune_Rev Build'!U18*'Neptune_Rev Build'!U19)*12*'Neptune COGS+OPEX Build'!$E$171)/1000000</f>
+        <f>(AVERAGE('Company Name Rev Build'!Q7,'Company Name Rev Build'!U7)*('Company Name Rev Build'!U18*'Company Name Rev Build'!U19)*12*'Company Name COGS+OPEX Build'!$E$171)/1000000</f>
         <v>8.1000648</v>
       </c>
       <c r="Q171">
-        <f>(AVERAGE('Neptune_Rev Build'!U7,'Neptune_Rev Build'!Y7)*('Neptune_Rev Build'!Y18*'Neptune_Rev Build'!Y19)*12*'Neptune COGS+OPEX Build'!$E$171)/1000000</f>
+        <f>(AVERAGE('Company Name Rev Build'!U7,'Company Name Rev Build'!Y7)*('Company Name Rev Build'!Y18*'Company Name Rev Build'!Y19)*12*'Company Name COGS+OPEX Build'!$E$171)/1000000</f>
         <v>11.3400648</v>
       </c>
       <c r="R171">
-        <f>(AVERAGE('Neptune_Rev Build'!Y7,'Neptune_Rev Build'!AC7)*('Neptune_Rev Build'!AC18*'Neptune_Rev Build'!AC19)*12*'Neptune COGS+OPEX Build'!$E$171)/1000000</f>
+        <f>(AVERAGE('Company Name Rev Build'!Y7,'Company Name Rev Build'!AC7)*('Company Name Rev Build'!AC18*'Company Name Rev Build'!AC19)*12*'Company Name COGS+OPEX Build'!$E$171)/1000000</f>
         <v>14.5800648</v>
       </c>
     </row>
@@ -10455,23 +10455,23 @@
         <v>0</v>
       </c>
       <c r="N172">
-        <f>$E$172*'Neptune_Rev Build'!M6*'Neptune COGS+OPEX Build'!$D$172/1000000</f>
+        <f>$E$172*'Company Name Rev Build'!M6*'Company Name COGS+OPEX Build'!$D$172/1000000</f>
         <v>0.67</v>
       </c>
       <c r="O172">
-        <f>$E$172*'Neptune_Rev Build'!Q6*'Neptune COGS+OPEX Build'!$D$172/1000000</f>
+        <f>$E$172*'Company Name Rev Build'!Q6*'Company Name COGS+OPEX Build'!$D$172/1000000</f>
         <v>0.67</v>
       </c>
       <c r="P172">
-        <f>$E$172*'Neptune_Rev Build'!U6*'Neptune COGS+OPEX Build'!$D$172/1000000</f>
+        <f>$E$172*'Company Name Rev Build'!U6*'Company Name COGS+OPEX Build'!$D$172/1000000</f>
         <v>0.67</v>
       </c>
       <c r="Q172">
-        <f>$E$172*'Neptune_Rev Build'!Y6*'Neptune COGS+OPEX Build'!$D$172/1000000</f>
+        <f>$E$172*'Company Name Rev Build'!Y6*'Company Name COGS+OPEX Build'!$D$172/1000000</f>
         <v>0.67</v>
       </c>
       <c r="R172">
-        <f>$E$172*'Neptune_Rev Build'!AC6*'Neptune COGS+OPEX Build'!$D$172/1000000</f>
+        <f>$E$172*'Company Name Rev Build'!AC6*'Company Name COGS+OPEX Build'!$D$172/1000000</f>
         <v>0.67</v>
       </c>
     </row>
@@ -10486,23 +10486,23 @@
         <v>0.1</v>
       </c>
       <c r="N173">
-        <f>('Neptune_Rev Build'!O23+'Neptune_Rev Build'!O31)*$E$173/1000</f>
+        <f>('Company Name Rev Build'!O23+'Company Name Rev Build'!O31)*$E$173/1000</f>
         <v>0.11389360799999998</v>
       </c>
       <c r="O173">
-        <f>('Neptune_Rev Build'!S23+'Neptune_Rev Build'!S31)*$E$173/1000</f>
+        <f>('Company Name Rev Build'!S23+'Company Name Rev Build'!S31)*$E$173/1000</f>
         <v>0.390831408</v>
       </c>
       <c r="P173">
-        <f>('Neptune_Rev Build'!W23+'Neptune_Rev Build'!W31)*$E$173/1000</f>
+        <f>('Company Name Rev Build'!W23+'Company Name Rev Build'!W31)*$E$173/1000</f>
         <v>0.6734465279999999</v>
       </c>
       <c r="Q173">
-        <f>('Neptune_Rev Build'!AA23+'Neptune_Rev Build'!AA31)*$E$173/1000</f>
+        <f>('Company Name Rev Build'!AA23+'Company Name Rev Build'!AA31)*$E$173/1000</f>
         <v>0.979632048</v>
       </c>
       <c r="R173">
-        <f>('Neptune_Rev Build'!AE23+'Neptune_Rev Build'!AE31)*$E$173/1000</f>
+        <f>('Company Name Rev Build'!AE23+'Company Name Rev Build'!AE31)*$E$173/1000</f>
         <v>1.309387968</v>
       </c>
     </row>
@@ -10517,23 +10517,23 @@
         <v>0.8</v>
       </c>
       <c r="N174">
-        <f>$E$174*'Neptune_Rev Build'!O12/1000000</f>
+        <f>$E$174*'Company Name Rev Build'!O12/1000000</f>
         <v>1.6915</v>
       </c>
       <c r="O174">
-        <f>$E$174*'Neptune_Rev Build'!S12/1000000</f>
+        <f>$E$174*'Company Name Rev Build'!S12/1000000</f>
         <v>2.1165</v>
       </c>
       <c r="P174">
-        <f>$E$174*'Neptune_Rev Build'!W12/1000000</f>
+        <f>$E$174*'Company Name Rev Build'!W12/1000000</f>
         <v>2.5415</v>
       </c>
       <c r="Q174">
-        <f>$E$174*'Neptune_Rev Build'!AA12/1000000</f>
+        <f>$E$174*'Company Name Rev Build'!AA12/1000000</f>
         <v>2.9665</v>
       </c>
       <c r="R174">
-        <f>$E$174*'Neptune_Rev Build'!AE12/1000000</f>
+        <f>$E$174*'Company Name Rev Build'!AE12/1000000</f>
         <v>3.3915</v>
       </c>
     </row>
@@ -10551,23 +10551,23 @@
         <v>0.159</v>
       </c>
       <c r="N175">
-        <f>('Neptune_Rev Build'!I10*87000/7+AVERAGE('Neptune_Rev Build'!M9,'Neptune_Rev Build'!M6)*'Neptune COGS+OPEX Build'!D176/7)/1000000</f>
+        <f>('Company Name Rev Build'!I10*87000/7+AVERAGE('Company Name Rev Build'!M9,'Company Name Rev Build'!M6)*'Company Name COGS+OPEX Build'!D176/7)/1000000</f>
         <v>0.8440714285714286</v>
       </c>
       <c r="O175">
-        <f>('Neptune_Rev Build'!M10*D176/7+AVERAGE('Neptune_Rev Build'!Q9,'Neptune_Rev Build'!Q6)*E176/7)/1000000</f>
+        <f>('Company Name Rev Build'!M10*D176/7+AVERAGE('Company Name Rev Build'!Q9,'Company Name Rev Build'!Q6)*E176/7)/1000000</f>
         <v>1.6622142857142856</v>
       </c>
       <c r="P175">
-        <f>('Neptune_Rev Build'!Q10*E176/7+AVERAGE('Neptune_Rev Build'!U9,'Neptune_Rev Build'!U6)*E176/7)/1000000</f>
+        <f>('Company Name Rev Build'!Q10*E176/7+AVERAGE('Company Name Rev Build'!U9,'Company Name Rev Build'!U6)*E176/7)/1000000</f>
         <v>2.5542857142857147</v>
       </c>
       <c r="Q175">
-        <f>('Neptune_Rev Build'!U10*E176/7+AVERAGE('Neptune_Rev Build'!Y9,'Neptune_Rev Build'!Y6)*E176/7)/1000000</f>
+        <f>('Company Name Rev Build'!U10*E176/7+AVERAGE('Company Name Rev Build'!Y9,'Company Name Rev Build'!Y6)*E176/7)/1000000</f>
         <v>3.8828571428571426</v>
       </c>
       <c r="R175">
-        <f>('Neptune_Rev Build'!Y10*E176/7+AVERAGE('Neptune_Rev Build'!AC9,'Neptune_Rev Build'!AC6)*E176/7)/1000000</f>
+        <f>('Company Name Rev Build'!Y10*E176/7+AVERAGE('Company Name Rev Build'!AC9,'Company Name Rev Build'!AC6)*E176/7)/1000000</f>
         <v>5.468571428571429</v>
       </c>
     </row>
@@ -10586,23 +10586,23 @@
         <v>0.312</v>
       </c>
       <c r="N176">
-        <f>$D$176*'Neptune_Rev Build'!O12/1000000</f>
+        <f>$D$176*'Company Name Rev Build'!O12/1000000</f>
         <v>14.6265</v>
       </c>
       <c r="O176">
-        <f>$E$176*'Neptune_Rev Build'!S12/1000000</f>
+        <f>$E$176*'Company Name Rev Build'!S12/1000000</f>
         <v>14.94</v>
       </c>
       <c r="P176">
-        <f>$E$176*'Neptune_Rev Build'!W12/1000000</f>
+        <f>$E$176*'Company Name Rev Build'!W12/1000000</f>
         <v>17.94</v>
       </c>
       <c r="Q176">
-        <f>$E$176*'Neptune_Rev Build'!AA12/1000000</f>
+        <f>$E$176*'Company Name Rev Build'!AA12/1000000</f>
         <v>20.94</v>
       </c>
       <c r="R176">
-        <f>$E$176*'Neptune_Rev Build'!AE12/1000000</f>
+        <f>$E$176*'Company Name Rev Build'!AE12/1000000</f>
         <v>23.94</v>
       </c>
     </row>
@@ -10774,27 +10774,27 @@
         <v>Product Rev.</v>
       </c>
       <c r="M183">
-        <f>SUM('Neptune_Rev Build'!K36,'Neptune_Rev Build'!K39)/1000</f>
+        <f>SUM('Company Name Rev Build'!K36,'Company Name Rev Build'!K39)/1000</f>
         <v>0.4969159999999999</v>
       </c>
       <c r="N183">
-        <f>SUM('Neptune_Rev Build'!O36,'Neptune_Rev Build'!O39)/1000</f>
+        <f>SUM('Company Name Rev Build'!O36,'Company Name Rev Build'!O39)/1000</f>
         <v>37.869360799999995</v>
       </c>
       <c r="O183">
-        <f>SUM('Neptune_Rev Build'!S36,'Neptune_Rev Build'!S39)/1000</f>
+        <f>SUM('Company Name Rev Build'!S36,'Company Name Rev Build'!S39)/1000</f>
         <v>75.0431408</v>
       </c>
       <c r="P183">
-        <f>SUM('Neptune_Rev Build'!W36,'Neptune_Rev Build'!W39)/1000</f>
+        <f>SUM('Company Name Rev Build'!W36,'Company Name Rev Build'!W39)/1000</f>
         <v>112.77165280000001</v>
       </c>
       <c r="Q183">
-        <f>SUM('Neptune_Rev Build'!AA36,'Neptune_Rev Build'!AA39)/1000</f>
+        <f>SUM('Company Name Rev Build'!AA36,'Company Name Rev Build'!AA39)/1000</f>
         <v>153.6372048</v>
       </c>
       <c r="R183">
-        <f>SUM('Neptune_Rev Build'!AE36,'Neptune_Rev Build'!AE39)/1000</f>
+        <f>SUM('Company Name Rev Build'!AE36,'Company Name Rev Build'!AE39)/1000</f>
         <v>197.6397968</v>
       </c>
     </row>
@@ -11038,27 +11038,27 @@
         <v>USARAD Rev.</v>
       </c>
       <c r="M193">
-        <f>SUM('Neptune_Rev Build'!K55,'Neptune_Rev Build'!K45)/1000</f>
+        <f>SUM('Company Name Rev Build'!K55,'Company Name Rev Build'!K45)/1000</f>
         <v>10.532</v>
       </c>
       <c r="N193">
-        <f>SUM('Neptune_Rev Build'!O45,'Neptune_Rev Build'!O55)/1000</f>
+        <f>SUM('Company Name Rev Build'!O45,'Company Name Rev Build'!O55)/1000</f>
         <v>12.673</v>
       </c>
       <c r="O193">
-        <f>SUM('Neptune_Rev Build'!S45,'Neptune_Rev Build'!S55)/1000</f>
+        <f>SUM('Company Name Rev Build'!S45,'Company Name Rev Build'!S55)/1000</f>
         <v>13.898</v>
       </c>
       <c r="P193">
-        <f>SUM('Neptune_Rev Build'!W45,'Neptune_Rev Build'!W55)/1000</f>
+        <f>SUM('Company Name Rev Build'!W45,'Company Name Rev Build'!W55)/1000</f>
         <v>15.29175</v>
       </c>
       <c r="Q193">
-        <f>SUM('Neptune_Rev Build'!AA45,'Neptune_Rev Build'!AA55)/1000</f>
+        <f>SUM('Company Name Rev Build'!AA45,'Company Name Rev Build'!AA55)/1000</f>
         <v>16.9808125</v>
       </c>
       <c r="R193">
-        <f>SUM('Neptune_Rev Build'!AE45,'Neptune_Rev Build'!AE55)/1000</f>
+        <f>SUM('Company Name Rev Build'!AE45,'Company Name Rev Build'!AE55)/1000</f>
         <v>19.186671875</v>
       </c>
     </row>
@@ -11581,7 +11581,7 @@
         <v>127379.31034482758</v>
       </c>
       <c r="F5">
-        <f>'Neptune_Rev Build'!Q12</f>
+        <f>'Company Name Rev Build'!Q12</f>
         <v>175</v>
       </c>
       <c r="H5">
@@ -11589,7 +11589,7 @@
         <v>126685.71428571429</v>
       </c>
       <c r="J5">
-        <f>'Neptune_Rev Build'!U12</f>
+        <f>'Company Name Rev Build'!U12</f>
         <v>205</v>
       </c>
       <c r="L5">
@@ -11597,7 +11597,7 @@
         <v>126658.53658536586</v>
       </c>
       <c r="N5">
-        <f>'Neptune_Rev Build'!Y12</f>
+        <f>'Company Name Rev Build'!Y12</f>
         <v>235</v>
       </c>
       <c r="P5">
@@ -11605,7 +11605,7 @@
         <v>126638.29787234042</v>
       </c>
       <c r="R5">
-        <f>'Neptune_Rev Build'!AC12</f>
+        <f>'Company Name Rev Build'!AC12</f>
         <v>265</v>
       </c>
       <c r="T5">
@@ -11701,7 +11701,7 @@
         <v>143555.55555555556</v>
       </c>
       <c r="F9">
-        <f>'Neptune_Rev Build'!R12</f>
+        <f>'Company Name Rev Build'!R12</f>
         <v>74</v>
       </c>
       <c r="H9">
@@ -11709,7 +11709,7 @@
         <v>160000</v>
       </c>
       <c r="J9">
-        <f>'Neptune_Rev Build'!V12</f>
+        <f>'Company Name Rev Build'!V12</f>
         <v>94</v>
       </c>
       <c r="L9">
@@ -11717,7 +11717,7 @@
         <v>160000</v>
       </c>
       <c r="N9">
-        <f>'Neptune_Rev Build'!Z12</f>
+        <f>'Company Name Rev Build'!Z12</f>
         <v>114</v>
       </c>
       <c r="P9">
@@ -11725,7 +11725,7 @@
         <v>160000</v>
       </c>
       <c r="R9">
-        <f>'Neptune_Rev Build'!AD12</f>
+        <f>'Company Name Rev Build'!AD12</f>
         <v>134</v>
       </c>
       <c r="T9">

</xml_diff>